<commit_message>
Schedule change: Days 1-3 Wed 14 to Fri 16 Oct, weekend rest, Days 4-7 Mon 19 to Thu 22 Oct; remove CIBN attribution
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/website/materials/Sahel_Sun_Capital_Stack_Template.xlsx
+++ b/website/materials/Sahel_Sun_Capital_Stack_Template.xlsx
@@ -78,13 +78,13 @@
     <t>solar IPP, not taken from any actual transaction. Market reference points used: CBN MPR 26.5% (MPC, July 2026); CBN USD/NGN ≈ 1,330 (Sept 2026).</t>
   </si>
   <si>
-    <t>Mastering Infrastructure and Project Finance (MIPF) Boot Camp  |  Lagos Business School  |  14 to 21 October 2026</t>
+    <t>Mastering Infrastructure and Project Finance (MIPF) Boot Camp  |  Lagos Business School  |  14 to 22 October 2026</t>
   </si>
   <si>
     <t>Prof Bongo Adi  |  +234 706 164 8699  |  badi@lbs.edu.ng  |  bongo.adi@fulbrightmail.org</t>
   </si>
   <si>
-    <t>Adapted from the CIBN Centre for Financial Studies workshop (facilitator: Prof. Bongo Adi). Teaching case; all figures illustrative.</t>
+    <t>Teaching case; all figures illustrative.</t>
   </si>
   <si>
     <t>Inputs &amp; Assumptions</t>

</xml_diff>